<commit_message>
ingesta: snapshot 2026-07-31 18:49 UTC
</commit_message>
<xml_diff>
--- a/data_lake/datos_diarios_preliminares/dt=2026-07-31/CORDOBA_JUL26.xlsx
+++ b/data_lake/datos_diarios_preliminares/dt=2026-07-31/CORDOBA_JUL26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B2EA829-CCD3-4ED2-84AF-4CF55AC36E71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0928799E-C53D-4B03-A96D-17AB914E1650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="2205" windowWidth="21600" windowHeight="11295" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
   </bookViews>
   <sheets>
     <sheet name="ENERO_2026" sheetId="1" r:id="rId1"/>
@@ -7393,7 +7393,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7866,7 +7866,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -8470,7 +8470,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -9079,7 +9079,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -9689,7 +9689,7 @@
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -10047,7 +10047,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>-1</c:v>
+                  <c:v>88.7</c:v>
                 </c:pt>
                 <c:pt idx="30">
                   <c:v>-1</c:v>
@@ -20006,7 +20006,9 @@
       <c r="AG3" s="25">
         <v>0</v>
       </c>
-      <c r="AH3" s="25"/>
+      <c r="AH3" s="25">
+        <v>0</v>
+      </c>
       <c r="AI3" s="34"/>
       <c r="AJ3" s="36">
         <f>SUM(E3:AI3)</f>
@@ -20116,7 +20118,9 @@
       <c r="AG4" s="25">
         <v>0</v>
       </c>
-      <c r="AH4" s="25"/>
+      <c r="AH4" s="25">
+        <v>0</v>
+      </c>
       <c r="AI4" s="34"/>
       <c r="AJ4" s="36">
         <f t="shared" ref="AJ4:AJ17" si="0">SUM(E4:AI4)</f>
@@ -20226,11 +20230,13 @@
       <c r="AG5" s="25">
         <v>0</v>
       </c>
-      <c r="AH5" s="25"/>
+      <c r="AH5" s="25">
+        <v>52</v>
+      </c>
       <c r="AI5" s="34"/>
       <c r="AJ5" s="36">
         <f t="shared" si="0"/>
-        <v>334.9</v>
+        <v>386.9</v>
       </c>
       <c r="AK5" s="30">
         <v>40.986206896551728</v>
@@ -20336,11 +20342,13 @@
       <c r="AG6" s="25">
         <v>0</v>
       </c>
-      <c r="AH6" s="25"/>
+      <c r="AH6" s="25">
+        <v>3.7</v>
+      </c>
       <c r="AI6" s="34"/>
       <c r="AJ6" s="36">
         <f t="shared" si="0"/>
-        <v>142.70000000000002</v>
+        <v>146.4</v>
       </c>
       <c r="AK6" s="30">
         <v>88.719230769230762</v>
@@ -20550,11 +20558,13 @@
       <c r="AG9" s="25">
         <v>0</v>
       </c>
-      <c r="AH9" s="25"/>
+      <c r="AH9" s="25">
+        <v>33</v>
+      </c>
       <c r="AI9" s="34"/>
       <c r="AJ9" s="36">
         <f t="shared" si="0"/>
-        <v>119</v>
+        <v>152</v>
       </c>
       <c r="AK9" s="30">
         <v>65.482758620689651</v>
@@ -20738,7 +20748,9 @@
       <c r="AG11" s="25">
         <v>0</v>
       </c>
-      <c r="AH11" s="25"/>
+      <c r="AH11" s="25">
+        <v>0</v>
+      </c>
       <c r="AI11" s="34"/>
       <c r="AJ11" s="36">
         <f t="shared" si="0"/>
@@ -20846,7 +20858,9 @@
       <c r="AG12" s="25">
         <v>0</v>
       </c>
-      <c r="AH12" s="25"/>
+      <c r="AH12" s="25">
+        <v>0</v>
+      </c>
       <c r="AI12" s="34"/>
       <c r="AJ12" s="36">
         <f t="shared" si="0"/>
@@ -20956,7 +20970,9 @@
       <c r="AG13" s="25">
         <v>0</v>
       </c>
-      <c r="AH13" s="25"/>
+      <c r="AH13" s="25">
+        <v>0</v>
+      </c>
       <c r="AI13" s="34"/>
       <c r="AJ13" s="36">
         <f t="shared" si="0"/>
@@ -21064,7 +21080,9 @@
       <c r="AG14" s="25">
         <v>0</v>
       </c>
-      <c r="AH14" s="25"/>
+      <c r="AH14" s="25">
+        <v>0</v>
+      </c>
       <c r="AI14" s="34"/>
       <c r="AJ14" s="36">
         <f>SUM(E14:AI14)</f>
@@ -21174,7 +21192,9 @@
       <c r="AG15" s="25">
         <v>0</v>
       </c>
-      <c r="AH15" s="25"/>
+      <c r="AH15" s="25">
+        <v>0</v>
+      </c>
       <c r="AI15" s="34"/>
       <c r="AJ15" s="36">
         <f t="shared" si="0"/>
@@ -21404,7 +21424,7 @@
       </c>
       <c r="AH19" s="26">
         <f t="shared" si="1"/>
-        <v>-1</v>
+        <v>88.7</v>
       </c>
       <c r="AI19" s="26">
         <f t="shared" si="1"/>

</xml_diff>